<commit_message>
fix: rebuild processed layer so build_release runs first
The previous commit edited scripts and rebuilt downstream files but skipped
scripts/build_release.py, which generates entities.csv/entity_names.csv/
aliases.csv and back-fills the source_id provenance field. The new
guohan sources (SRC-GUOHAN-1989-43 for Rizhao, SRC-GUOHAN-1991-84 for
Chaozhou/Jieyang) are therefore now correctly attributed in entities and
in the derived roster. This rebuild runs the full CI order (build_release
first) so the committed processed files match what CI regenerates.

Diff is entirely source_id attribution changes for the three 1989-91
entities; no name/status/geometry drift. validate_data 10/10 PASS,
pytest 20/20.
</commit_message>
<xml_diff>
--- a/data/releases/v4.0/china_city_entity_master_V4.0.xlsx
+++ b/data/releases/v4.0/china_city_entity_master_V4.0.xlsx
@@ -11091,7 +11091,7 @@
         </is>
       </c>
       <c r="O146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P146" t="inlineStr"/>
       <c r="Q146" t="inlineStr"/>
@@ -16124,7 +16124,7 @@
         </is>
       </c>
       <c r="O215" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P215" t="inlineStr"/>
       <c r="Q215" t="inlineStr"/>
@@ -16197,7 +16197,7 @@
         </is>
       </c>
       <c r="O216" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P216" t="inlineStr"/>
       <c r="Q216" t="inlineStr"/>

</xml_diff>

<commit_message>
fix: capture all prefecture-level upgrades previously missed by the extractor
Full-coverage sweep found 10 prefecture events that existed in the
Wikipedia row archive but were never extracted, because the extractor's
patterns did not cover these sentence forms:
- '将东莞市升格为地级市' / '贵港市升格为地级市' (升格为, not 升为)
- '撤销县级泰州市，设立地级泰州市' (地级X市, not 地级市)

Newly captured (all previously missing, all reviewed-verified):
1987 威海/三亚 upgrade; 1988 东莞/中山/大庸(→张家界, manual link)
upgrade; 1992 莱芜 upgrade; 1994 云浮; 1995 贵港; 1996 泰州/宿迁.

Event type refined: same-name establishment of a county-level city as
prefecture-level is an upgrade (automatic_continuity=true); '地级市'
is excluded as a candidate city name. Entry-direction gap detector now
reports 0 missing events across the whole roster (previously 6).

normalized events 94->104, unified 157->167. validate_data 10/10,
pytest 20/20 (one test made semantic instead of id-based).
</commit_message>
<xml_diff>
--- a/data/releases/v4.0/china_city_entity_master_V4.0.xlsx
+++ b/data/releases/v4.0/china_city_entity_master_V4.0.xlsx
@@ -6715,7 +6715,7 @@
         </is>
       </c>
       <c r="O86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P86" t="inlineStr"/>
       <c r="Q86" t="inlineStr"/>
@@ -6788,7 +6788,7 @@
         </is>
       </c>
       <c r="O87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P87" t="inlineStr"/>
       <c r="Q87" t="inlineStr"/>
@@ -11018,7 +11018,7 @@
         </is>
       </c>
       <c r="O145" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P145" t="inlineStr"/>
       <c r="Q145" t="inlineStr"/>
@@ -11160,7 +11160,7 @@
         </is>
       </c>
       <c r="O147" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P147" t="inlineStr"/>
       <c r="Q147" t="inlineStr"/>
@@ -14299,7 +14299,7 @@
         </is>
       </c>
       <c r="O190" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P190" t="inlineStr"/>
       <c r="Q190" t="inlineStr"/>
@@ -15978,7 +15978,7 @@
         </is>
       </c>
       <c r="O213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P213" t="inlineStr"/>
       <c r="Q213" t="inlineStr"/>
@@ -16051,7 +16051,7 @@
         </is>
       </c>
       <c r="O214" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P214" t="inlineStr"/>
       <c r="Q214" t="inlineStr"/>
@@ -16270,7 +16270,7 @@
         </is>
       </c>
       <c r="O217" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P217" t="inlineStr"/>
       <c r="Q217" t="inlineStr"/>
@@ -16854,7 +16854,7 @@
         </is>
       </c>
       <c r="O225" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P225" t="inlineStr"/>
       <c r="Q225" t="inlineStr"/>
@@ -17438,7 +17438,7 @@
         </is>
       </c>
       <c r="O233" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P233" t="inlineStr"/>
       <c r="Q233" t="inlineStr"/>

</xml_diff>